<commit_message>
[HUMAN-VALIDATION]: Incresed human validation tests done.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/01_REVISIONE_TEST_SET.xlsx
+++ b/thesis_evidence/validazione_umana/01_REVISIONE_TEST_SET.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="193">
   <si>
     <t xml:space="preserve">Revisione manuale dei 50 casi di test</t>
   </si>
@@ -422,6 +422,9 @@
   </si>
   <si>
     <t xml:space="preserve">Flag cartFailure attivato, variante 100%. AddItem HTTP 200; checkout HTTP 504. cart / POST /oteldemo.CartService/EmptyCart: stato ERROR, durata 112267.5 ms. cart / POST /oteldemo.CartService/EmptyCart: stato ERROR, durata 112267.5 ms. Traccia normalizzata: 44 span, 3 in errore.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo scenario, la causa e la risposta attesa sono coerenti; incident_context ripete lo span Cart e deve riportare anche lo span client di Checkout. La cattura di test -03 non è inclusa come file grezzo negli input minimi.</t>
   </si>
   <si>
     <t xml:space="preserve">test_product_catalog_failure_01</t>
@@ -1226,8 +1229,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="n">
-        <f aca="false">COUNTIF(T9:T58,"OK")</f>
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1936,17 +1938,31 @@
       <c r="K19" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L19" s="15"/>
-      <c r="M19" s="15"/>
-      <c r="N19" s="15"/>
-      <c r="O19" s="15"/>
-      <c r="P19" s="15"/>
-      <c r="Q19" s="15"/>
+      <c r="L19" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M19" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N19" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O19" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P19" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q19" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R19" s="15"/>
-      <c r="S19" s="15"/>
+      <c r="S19" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T19" s="16" t="str">
         <f aca="false">IF(AND(L19&lt;&gt;"",M19&lt;&gt;"",N19&lt;&gt;"",O19&lt;&gt;"",P19&lt;&gt;"",Q19&lt;&gt;"",OR(L19&lt;&gt;"CORREGGERE",R19&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1983,17 +1999,31 @@
       <c r="K20" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
+      <c r="L20" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M20" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N20" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O20" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P20" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R20" s="15"/>
-      <c r="S20" s="15"/>
+      <c r="S20" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T20" s="16" t="str">
         <f aca="false">IF(AND(L20&lt;&gt;"",M20&lt;&gt;"",N20&lt;&gt;"",O20&lt;&gt;"",P20&lt;&gt;"",Q20&lt;&gt;"",OR(L20&lt;&gt;"CORREGGERE",R20&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2030,17 +2060,31 @@
       <c r="K21" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15"/>
-      <c r="N21" s="15"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-      <c r="Q21" s="15"/>
+      <c r="L21" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M21" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N21" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O21" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P21" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q21" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R21" s="15"/>
-      <c r="S21" s="15"/>
+      <c r="S21" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T21" s="16" t="str">
         <f aca="false">IF(AND(L21&lt;&gt;"",M21&lt;&gt;"",N21&lt;&gt;"",O21&lt;&gt;"",P21&lt;&gt;"",Q21&lt;&gt;"",OR(L21&lt;&gt;"CORREGGERE",R21&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2077,17 +2121,31 @@
       <c r="K22" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15"/>
-      <c r="Q22" s="15"/>
+      <c r="L22" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M22" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N22" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O22" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P22" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q22" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R22" s="15"/>
-      <c r="S22" s="15"/>
+      <c r="S22" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T22" s="16" t="str">
         <f aca="false">IF(AND(L22&lt;&gt;"",M22&lt;&gt;"",N22&lt;&gt;"",O22&lt;&gt;"",P22&lt;&gt;"",Q22&lt;&gt;"",OR(L22&lt;&gt;"CORREGGERE",R22&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2124,17 +2182,31 @@
       <c r="K23" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
-      <c r="N23" s="15"/>
-      <c r="O23" s="15"/>
-      <c r="P23" s="15"/>
-      <c r="Q23" s="15"/>
+      <c r="L23" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M23" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N23" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O23" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P23" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q23" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R23" s="15"/>
-      <c r="S23" s="15"/>
+      <c r="S23" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T23" s="16" t="str">
         <f aca="false">IF(AND(L23&lt;&gt;"",M23&lt;&gt;"",N23&lt;&gt;"",O23&lt;&gt;"",P23&lt;&gt;"",Q23&lt;&gt;"",OR(L23&lt;&gt;"CORREGGERE",R23&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2171,17 +2243,31 @@
       <c r="K24" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L24" s="15"/>
-      <c r="M24" s="15"/>
-      <c r="N24" s="15"/>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
+      <c r="L24" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M24" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N24" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O24" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P24" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q24" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R24" s="15"/>
-      <c r="S24" s="15"/>
+      <c r="S24" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T24" s="16" t="str">
         <f aca="false">IF(AND(L24&lt;&gt;"",M24&lt;&gt;"",N24&lt;&gt;"",O24&lt;&gt;"",P24&lt;&gt;"",Q24&lt;&gt;"",OR(L24&lt;&gt;"CORREGGERE",R24&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2218,17 +2304,31 @@
       <c r="K25" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
+      <c r="L25" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M25" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N25" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O25" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P25" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q25" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R25" s="15"/>
-      <c r="S25" s="15"/>
+      <c r="S25" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T25" s="16" t="str">
         <f aca="false">IF(AND(L25&lt;&gt;"",M25&lt;&gt;"",N25&lt;&gt;"",O25&lt;&gt;"",P25&lt;&gt;"",Q25&lt;&gt;"",OR(L25&lt;&gt;"CORREGGERE",R25&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2265,17 +2365,31 @@
       <c r="K26" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="15"/>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="15"/>
+      <c r="L26" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M26" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N26" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O26" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P26" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q26" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R26" s="15"/>
-      <c r="S26" s="15"/>
+      <c r="S26" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T26" s="16" t="str">
         <f aca="false">IF(AND(L26&lt;&gt;"",M26&lt;&gt;"",N26&lt;&gt;"",O26&lt;&gt;"",P26&lt;&gt;"",Q26&lt;&gt;"",OR(L26&lt;&gt;"CORREGGERE",R26&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2312,17 +2426,31 @@
       <c r="K27" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L27" s="15"/>
-      <c r="M27" s="15"/>
-      <c r="N27" s="15"/>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="15"/>
+      <c r="L27" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M27" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N27" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O27" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P27" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q27" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R27" s="15"/>
-      <c r="S27" s="15"/>
+      <c r="S27" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T27" s="16" t="str">
         <f aca="false">IF(AND(L27&lt;&gt;"",M27&lt;&gt;"",N27&lt;&gt;"",O27&lt;&gt;"",P27&lt;&gt;"",Q27&lt;&gt;"",OR(L27&lt;&gt;"CORREGGERE",R27&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2359,17 +2487,31 @@
       <c r="K28" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
-      <c r="Q28" s="15"/>
+      <c r="L28" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M28" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N28" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O28" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P28" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q28" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R28" s="15"/>
-      <c r="S28" s="15"/>
+      <c r="S28" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T28" s="16" t="str">
         <f aca="false">IF(AND(L28&lt;&gt;"",M28&lt;&gt;"",N28&lt;&gt;"",O28&lt;&gt;"",P28&lt;&gt;"",Q28&lt;&gt;"",OR(L28&lt;&gt;"CORREGGERE",R28&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2406,17 +2548,31 @@
       <c r="K29" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="15"/>
+      <c r="L29" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M29" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N29" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O29" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P29" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q29" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R29" s="15"/>
-      <c r="S29" s="15"/>
+      <c r="S29" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T29" s="16" t="str">
         <f aca="false">IF(AND(L29&lt;&gt;"",M29&lt;&gt;"",N29&lt;&gt;"",O29&lt;&gt;"",P29&lt;&gt;"",Q29&lt;&gt;"",OR(L29&lt;&gt;"CORREGGERE",R29&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2453,17 +2609,31 @@
       <c r="K30" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-      <c r="N30" s="15"/>
-      <c r="O30" s="15"/>
-      <c r="P30" s="15"/>
-      <c r="Q30" s="15"/>
+      <c r="L30" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M30" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N30" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O30" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P30" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q30" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R30" s="15"/>
-      <c r="S30" s="15"/>
+      <c r="S30" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T30" s="16" t="str">
         <f aca="false">IF(AND(L30&lt;&gt;"",M30&lt;&gt;"",N30&lt;&gt;"",O30&lt;&gt;"",P30&lt;&gt;"",Q30&lt;&gt;"",OR(L30&lt;&gt;"CORREGGERE",R30&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2500,17 +2670,31 @@
       <c r="K31" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="15"/>
-      <c r="P31" s="15"/>
-      <c r="Q31" s="15"/>
+      <c r="L31" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M31" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N31" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O31" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P31" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q31" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R31" s="15"/>
-      <c r="S31" s="15"/>
+      <c r="S31" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T31" s="16" t="str">
         <f aca="false">IF(AND(L31&lt;&gt;"",M31&lt;&gt;"",N31&lt;&gt;"",O31&lt;&gt;"",P31&lt;&gt;"",Q31&lt;&gt;"",OR(L31&lt;&gt;"CORREGGERE",R31&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2547,17 +2731,31 @@
       <c r="K32" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
-      <c r="N32" s="15"/>
-      <c r="O32" s="15"/>
-      <c r="P32" s="15"/>
-      <c r="Q32" s="15"/>
+      <c r="L32" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M32" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N32" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O32" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P32" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q32" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R32" s="15"/>
-      <c r="S32" s="15"/>
+      <c r="S32" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T32" s="16" t="str">
         <f aca="false">IF(AND(L32&lt;&gt;"",M32&lt;&gt;"",N32&lt;&gt;"",O32&lt;&gt;"",P32&lt;&gt;"",Q32&lt;&gt;"",OR(L32&lt;&gt;"CORREGGERE",R32&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2594,17 +2792,31 @@
       <c r="K33" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
-      <c r="N33" s="15"/>
-      <c r="O33" s="15"/>
-      <c r="P33" s="15"/>
-      <c r="Q33" s="15"/>
+      <c r="L33" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M33" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N33" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O33" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P33" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q33" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R33" s="15"/>
-      <c r="S33" s="15"/>
+      <c r="S33" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T33" s="16" t="str">
         <f aca="false">IF(AND(L33&lt;&gt;"",M33&lt;&gt;"",N33&lt;&gt;"",O33&lt;&gt;"",P33&lt;&gt;"",Q33&lt;&gt;"",OR(L33&lt;&gt;"CORREGGERE",R33&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2641,17 +2853,31 @@
       <c r="K34" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
-      <c r="N34" s="15"/>
-      <c r="O34" s="15"/>
-      <c r="P34" s="15"/>
-      <c r="Q34" s="15"/>
+      <c r="L34" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M34" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N34" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O34" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P34" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q34" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R34" s="15"/>
-      <c r="S34" s="15"/>
+      <c r="S34" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T34" s="16" t="str">
         <f aca="false">IF(AND(L34&lt;&gt;"",M34&lt;&gt;"",N34&lt;&gt;"",O34&lt;&gt;"",P34&lt;&gt;"",Q34&lt;&gt;"",OR(L34&lt;&gt;"CORREGGERE",R34&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2688,17 +2914,31 @@
       <c r="K35" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="N35" s="15"/>
-      <c r="O35" s="15"/>
-      <c r="P35" s="15"/>
-      <c r="Q35" s="15"/>
+      <c r="L35" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M35" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N35" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O35" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P35" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q35" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R35" s="15"/>
-      <c r="S35" s="15"/>
+      <c r="S35" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T35" s="16" t="str">
         <f aca="false">IF(AND(L35&lt;&gt;"",M35&lt;&gt;"",N35&lt;&gt;"",O35&lt;&gt;"",P35&lt;&gt;"",Q35&lt;&gt;"",OR(L35&lt;&gt;"CORREGGERE",R35&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2735,17 +2975,31 @@
       <c r="K36" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L36" s="15"/>
-      <c r="M36" s="15"/>
-      <c r="N36" s="15"/>
-      <c r="O36" s="15"/>
-      <c r="P36" s="15"/>
-      <c r="Q36" s="15"/>
+      <c r="L36" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M36" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N36" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O36" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P36" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q36" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R36" s="15"/>
-      <c r="S36" s="15"/>
+      <c r="S36" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T36" s="16" t="str">
         <f aca="false">IF(AND(L36&lt;&gt;"",M36&lt;&gt;"",N36&lt;&gt;"",O36&lt;&gt;"",P36&lt;&gt;"",Q36&lt;&gt;"",OR(L36&lt;&gt;"CORREGGERE",R36&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2782,17 +3036,31 @@
       <c r="K37" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L37" s="15"/>
-      <c r="M37" s="15"/>
-      <c r="N37" s="15"/>
-      <c r="O37" s="15"/>
-      <c r="P37" s="15"/>
-      <c r="Q37" s="15"/>
+      <c r="L37" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M37" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N37" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O37" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P37" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q37" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R37" s="15"/>
-      <c r="S37" s="15"/>
+      <c r="S37" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T37" s="16" t="str">
         <f aca="false">IF(AND(L37&lt;&gt;"",M37&lt;&gt;"",N37&lt;&gt;"",O37&lt;&gt;"",P37&lt;&gt;"",Q37&lt;&gt;"",OR(L37&lt;&gt;"CORREGGERE",R37&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2829,25 +3097,39 @@
       <c r="K38" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="L38" s="15"/>
-      <c r="M38" s="15"/>
-      <c r="N38" s="15"/>
-      <c r="O38" s="15"/>
-      <c r="P38" s="15"/>
-      <c r="Q38" s="15"/>
+      <c r="L38" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M38" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N38" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O38" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P38" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q38" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R38" s="15"/>
-      <c r="S38" s="15"/>
+      <c r="S38" s="15" t="s">
+        <v>133</v>
+      </c>
       <c r="T38" s="16" t="str">
         <f aca="false">IF(AND(L38&lt;&gt;"",M38&lt;&gt;"",N38&lt;&gt;"",O38&lt;&gt;"",P38&lt;&gt;"",Q38&lt;&gt;"",OR(L38&lt;&gt;"CORREGGERE",R38&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C39" s="14" t="s">
         <v>29</v>
@@ -2856,25 +3138,25 @@
         <v>30</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I39" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J39" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K39" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -2891,10 +3173,10 @@
     </row>
     <row r="40" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C40" s="14" t="s">
         <v>42</v>
@@ -2903,25 +3185,25 @@
         <v>43</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I40" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J40" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K40" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15"/>
@@ -2938,10 +3220,10 @@
     </row>
     <row r="41" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C41" s="14" t="s">
         <v>42</v>
@@ -2950,25 +3232,25 @@
         <v>43</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F41" s="14" t="s">
         <v>47</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J41" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K41" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L41" s="15"/>
       <c r="M41" s="15"/>
@@ -2985,10 +3267,10 @@
     </row>
     <row r="42" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>50</v>
@@ -2997,25 +3279,25 @@
         <v>51</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F42" s="14" t="s">
         <v>52</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J42" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K42" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L42" s="15"/>
       <c r="M42" s="15"/>
@@ -3032,10 +3314,10 @@
     </row>
     <row r="43" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>50</v>
@@ -3044,25 +3326,25 @@
         <v>43</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F43" s="14" t="s">
         <v>55</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J43" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K43" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15"/>
@@ -3079,10 +3361,10 @@
     </row>
     <row r="44" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>50</v>
@@ -3091,25 +3373,25 @@
         <v>51</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F44" s="14" t="s">
         <v>59</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H44" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J44" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K44" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L44" s="15"/>
       <c r="M44" s="15"/>
@@ -3126,10 +3408,10 @@
     </row>
     <row r="45" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C45" s="14" t="s">
         <v>42</v>
@@ -3138,25 +3420,25 @@
         <v>43</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F45" s="14" t="s">
         <v>62</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H45" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K45" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L45" s="15"/>
       <c r="M45" s="15"/>
@@ -3173,10 +3455,10 @@
     </row>
     <row r="46" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>29</v>
@@ -3185,25 +3467,25 @@
         <v>51</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H46" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I46" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K46" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L46" s="15"/>
       <c r="M46" s="15"/>
@@ -3220,10 +3502,10 @@
     </row>
     <row r="47" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C47" s="14" t="s">
         <v>42</v>
@@ -3232,25 +3514,25 @@
         <v>43</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F47" s="14" t="s">
         <v>68</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I47" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K47" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L47" s="15"/>
       <c r="M47" s="15"/>
@@ -3267,10 +3549,10 @@
     </row>
     <row r="48" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>42</v>
@@ -3279,25 +3561,25 @@
         <v>43</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F48" s="14" t="s">
         <v>71</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H48" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J48" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K48" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L48" s="15"/>
       <c r="M48" s="15"/>
@@ -3314,10 +3596,10 @@
     </row>
     <row r="49" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C49" s="14" t="s">
         <v>29</v>
@@ -3326,25 +3608,25 @@
         <v>30</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J49" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K49" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L49" s="15"/>
       <c r="M49" s="15"/>
@@ -3361,10 +3643,10 @@
     </row>
     <row r="50" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C50" s="14" t="s">
         <v>42</v>
@@ -3373,25 +3655,25 @@
         <v>43</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I50" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J50" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L50" s="15"/>
       <c r="M50" s="15"/>
@@ -3408,10 +3690,10 @@
     </row>
     <row r="51" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C51" s="14" t="s">
         <v>42</v>
@@ -3420,25 +3702,25 @@
         <v>43</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F51" s="14" t="s">
         <v>47</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H51" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J51" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L51" s="15"/>
       <c r="M51" s="15"/>
@@ -3455,10 +3737,10 @@
     </row>
     <row r="52" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C52" s="14" t="s">
         <v>50</v>
@@ -3467,25 +3749,25 @@
         <v>51</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F52" s="14" t="s">
         <v>52</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I52" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L52" s="15"/>
       <c r="M52" s="15"/>
@@ -3502,10 +3784,10 @@
     </row>
     <row r="53" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C53" s="14" t="s">
         <v>50</v>
@@ -3514,25 +3796,25 @@
         <v>43</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F53" s="14" t="s">
         <v>55</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I53" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J53" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K53" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L53" s="15"/>
       <c r="M53" s="15"/>
@@ -3549,10 +3831,10 @@
     </row>
     <row r="54" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>50</v>
@@ -3561,25 +3843,25 @@
         <v>51</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F54" s="14" t="s">
         <v>59</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L54" s="15"/>
       <c r="M54" s="15"/>
@@ -3596,10 +3878,10 @@
     </row>
     <row r="55" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C55" s="14" t="s">
         <v>42</v>
@@ -3608,25 +3890,25 @@
         <v>43</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F55" s="14" t="s">
         <v>62</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I55" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L55" s="15"/>
       <c r="M55" s="15"/>
@@ -3643,10 +3925,10 @@
     </row>
     <row r="56" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C56" s="14" t="s">
         <v>29</v>
@@ -3655,25 +3937,25 @@
         <v>51</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H56" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I56" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L56" s="15"/>
       <c r="M56" s="15"/>
@@ -3690,10 +3972,10 @@
     </row>
     <row r="57" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C57" s="14" t="s">
         <v>42</v>
@@ -3702,25 +3984,25 @@
         <v>43</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F57" s="14" t="s">
         <v>68</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H57" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L57" s="15"/>
       <c r="M57" s="15"/>
@@ -3737,10 +4019,10 @@
     </row>
     <row r="58" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C58" s="14" t="s">
         <v>42</v>
@@ -3749,25 +4031,25 @@
         <v>43</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F58" s="14" t="s">
         <v>71</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I58" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L58" s="15"/>
       <c r="M58" s="15"/>

</xml_diff>

<commit_message>
[HUMAN-VALIDATION]: Increased human validation tests done.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/01_REVISIONE_TEST_SET.xlsx
+++ b/thesis_evidence/validazione_umana/01_REVISIONE_TEST_SET.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="194">
   <si>
     <t xml:space="preserve">Revisione manuale dei 50 casi di test</t>
   </si>
@@ -453,6 +453,9 @@
   </si>
   <si>
     <t xml:space="preserve">product-catalog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario e valori HTTP coerenti con il runbook. La correzione elimina il riferimento operativo alla patch e descrive la modifica temporanea della regola di targeting. La cattura di test -03 non è inclusa come file grezzo negli input minimi.</t>
   </si>
   <si>
     <t xml:space="preserve">test_product_catalog_failure_02</t>
@@ -1229,7 +1232,8 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>30</v>
+        <f aca="false">COUNTIF(T9:T58,"OK")</f>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3158,22 +3162,36 @@
       <c r="K39" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L39" s="15"/>
-      <c r="M39" s="15"/>
-      <c r="N39" s="15"/>
-      <c r="O39" s="15"/>
-      <c r="P39" s="15"/>
-      <c r="Q39" s="15"/>
+      <c r="L39" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M39" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N39" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O39" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P39" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q39" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R39" s="15"/>
-      <c r="S39" s="15"/>
+      <c r="S39" s="15" t="s">
+        <v>143</v>
+      </c>
       <c r="T39" s="16" t="str">
         <f aca="false">IF(AND(L39&lt;&gt;"",M39&lt;&gt;"",N39&lt;&gt;"",O39&lt;&gt;"",P39&lt;&gt;"",Q39&lt;&gt;"",OR(L39&lt;&gt;"CORREGGERE",R39&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>135</v>
@@ -3188,10 +3206,10 @@
         <v>136</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H40" s="14" t="s">
         <v>139</v>
@@ -3205,22 +3223,36 @@
       <c r="K40" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L40" s="15"/>
-      <c r="M40" s="15"/>
-      <c r="N40" s="15"/>
-      <c r="O40" s="15"/>
-      <c r="P40" s="15"/>
-      <c r="Q40" s="15"/>
+      <c r="L40" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M40" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N40" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O40" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P40" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q40" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R40" s="15"/>
-      <c r="S40" s="15"/>
+      <c r="S40" s="15" t="s">
+        <v>143</v>
+      </c>
       <c r="T40" s="16" t="str">
         <f aca="false">IF(AND(L40&lt;&gt;"",M40&lt;&gt;"",N40&lt;&gt;"",O40&lt;&gt;"",P40&lt;&gt;"",Q40&lt;&gt;"",OR(L40&lt;&gt;"CORREGGERE",R40&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>135</v>
@@ -3238,7 +3270,7 @@
         <v>47</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H41" s="14" t="s">
         <v>139</v>
@@ -3252,22 +3284,36 @@
       <c r="K41" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L41" s="15"/>
-      <c r="M41" s="15"/>
-      <c r="N41" s="15"/>
-      <c r="O41" s="15"/>
-      <c r="P41" s="15"/>
-      <c r="Q41" s="15"/>
+      <c r="L41" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M41" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N41" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O41" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P41" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q41" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R41" s="15"/>
-      <c r="S41" s="15"/>
+      <c r="S41" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T41" s="16" t="str">
         <f aca="false">IF(AND(L41&lt;&gt;"",M41&lt;&gt;"",N41&lt;&gt;"",O41&lt;&gt;"",P41&lt;&gt;"",Q41&lt;&gt;"",OR(L41&lt;&gt;"CORREGGERE",R41&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>135</v>
@@ -3285,7 +3331,7 @@
         <v>52</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H42" s="14" t="s">
         <v>139</v>
@@ -3299,22 +3345,36 @@
       <c r="K42" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L42" s="15"/>
-      <c r="M42" s="15"/>
-      <c r="N42" s="15"/>
-      <c r="O42" s="15"/>
-      <c r="P42" s="15"/>
-      <c r="Q42" s="15"/>
+      <c r="L42" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M42" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N42" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O42" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P42" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q42" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R42" s="15"/>
-      <c r="S42" s="15"/>
+      <c r="S42" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T42" s="16" t="str">
         <f aca="false">IF(AND(L42&lt;&gt;"",M42&lt;&gt;"",N42&lt;&gt;"",O42&lt;&gt;"",P42&lt;&gt;"",Q42&lt;&gt;"",OR(L42&lt;&gt;"CORREGGERE",R42&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>135</v>
@@ -3332,13 +3392,13 @@
         <v>55</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H43" s="14" t="s">
         <v>139</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J43" s="14" t="s">
         <v>141</v>
@@ -3346,22 +3406,36 @@
       <c r="K43" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L43" s="15"/>
-      <c r="M43" s="15"/>
-      <c r="N43" s="15"/>
-      <c r="O43" s="15"/>
-      <c r="P43" s="15"/>
-      <c r="Q43" s="15"/>
+      <c r="L43" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M43" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N43" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O43" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P43" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q43" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R43" s="15"/>
-      <c r="S43" s="15"/>
+      <c r="S43" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T43" s="16" t="str">
         <f aca="false">IF(AND(L43&lt;&gt;"",M43&lt;&gt;"",N43&lt;&gt;"",O43&lt;&gt;"",P43&lt;&gt;"",Q43&lt;&gt;"",OR(L43&lt;&gt;"CORREGGERE",R43&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>135</v>
@@ -3379,7 +3453,7 @@
         <v>59</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H44" s="14" t="s">
         <v>139</v>
@@ -3393,22 +3467,36 @@
       <c r="K44" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L44" s="15"/>
-      <c r="M44" s="15"/>
-      <c r="N44" s="15"/>
-      <c r="O44" s="15"/>
-      <c r="P44" s="15"/>
-      <c r="Q44" s="15"/>
+      <c r="L44" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M44" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N44" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O44" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P44" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q44" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R44" s="15"/>
-      <c r="S44" s="15"/>
+      <c r="S44" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T44" s="16" t="str">
         <f aca="false">IF(AND(L44&lt;&gt;"",M44&lt;&gt;"",N44&lt;&gt;"",O44&lt;&gt;"",P44&lt;&gt;"",Q44&lt;&gt;"",OR(L44&lt;&gt;"CORREGGERE",R44&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>135</v>
@@ -3426,7 +3514,7 @@
         <v>62</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H45" s="14" t="s">
         <v>139</v>
@@ -3440,22 +3528,36 @@
       <c r="K45" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L45" s="15"/>
-      <c r="M45" s="15"/>
-      <c r="N45" s="15"/>
-      <c r="O45" s="15"/>
-      <c r="P45" s="15"/>
-      <c r="Q45" s="15"/>
+      <c r="L45" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M45" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N45" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O45" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P45" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q45" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R45" s="15"/>
-      <c r="S45" s="15"/>
+      <c r="S45" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T45" s="16" t="str">
         <f aca="false">IF(AND(L45&lt;&gt;"",M45&lt;&gt;"",N45&lt;&gt;"",O45&lt;&gt;"",P45&lt;&gt;"",Q45&lt;&gt;"",OR(L45&lt;&gt;"CORREGGERE",R45&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>135</v>
@@ -3470,10 +3572,10 @@
         <v>136</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H46" s="14" t="s">
         <v>139</v>
@@ -3487,22 +3589,36 @@
       <c r="K46" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L46" s="15"/>
-      <c r="M46" s="15"/>
-      <c r="N46" s="15"/>
-      <c r="O46" s="15"/>
-      <c r="P46" s="15"/>
-      <c r="Q46" s="15"/>
+      <c r="L46" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M46" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N46" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O46" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P46" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q46" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R46" s="15"/>
-      <c r="S46" s="15"/>
+      <c r="S46" s="15" t="s">
+        <v>143</v>
+      </c>
       <c r="T46" s="16" t="str">
         <f aca="false">IF(AND(L46&lt;&gt;"",M46&lt;&gt;"",N46&lt;&gt;"",O46&lt;&gt;"",P46&lt;&gt;"",Q46&lt;&gt;"",OR(L46&lt;&gt;"CORREGGERE",R46&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>135</v>
@@ -3520,7 +3636,7 @@
         <v>68</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H47" s="14" t="s">
         <v>139</v>
@@ -3534,22 +3650,36 @@
       <c r="K47" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L47" s="15"/>
-      <c r="M47" s="15"/>
-      <c r="N47" s="15"/>
-      <c r="O47" s="15"/>
-      <c r="P47" s="15"/>
-      <c r="Q47" s="15"/>
+      <c r="L47" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M47" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N47" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O47" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P47" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q47" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R47" s="15"/>
-      <c r="S47" s="15"/>
+      <c r="S47" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="T47" s="16" t="str">
         <f aca="false">IF(AND(L47&lt;&gt;"",M47&lt;&gt;"",N47&lt;&gt;"",O47&lt;&gt;"",P47&lt;&gt;"",Q47&lt;&gt;"",OR(L47&lt;&gt;"CORREGGERE",R47&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>135</v>
@@ -3567,7 +3697,7 @@
         <v>71</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H48" s="14" t="s">
         <v>139</v>
@@ -3581,25 +3711,39 @@
       <c r="K48" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="L48" s="15"/>
-      <c r="M48" s="15"/>
-      <c r="N48" s="15"/>
-      <c r="O48" s="15"/>
-      <c r="P48" s="15"/>
-      <c r="Q48" s="15"/>
+      <c r="L48" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M48" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N48" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O48" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="P48" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q48" s="15" t="s">
+        <v>39</v>
+      </c>
       <c r="R48" s="15"/>
-      <c r="S48" s="15"/>
+      <c r="S48" s="15" t="s">
+        <v>143</v>
+      </c>
       <c r="T48" s="16" t="str">
         <f aca="false">IF(AND(L48&lt;&gt;"",M48&lt;&gt;"",N48&lt;&gt;"",O48&lt;&gt;"",P48&lt;&gt;"",Q48&lt;&gt;"",OR(L48&lt;&gt;"CORREGGERE",R48&lt;&gt;"")),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C49" s="14" t="s">
         <v>29</v>
@@ -3608,22 +3752,22 @@
         <v>30</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J49" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K49" s="14" t="s">
         <v>142</v>
@@ -3643,10 +3787,10 @@
     </row>
     <row r="50" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C50" s="14" t="s">
         <v>42</v>
@@ -3655,22 +3799,22 @@
         <v>43</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I50" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J50" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K50" s="14" t="s">
         <v>142</v>
@@ -3690,10 +3834,10 @@
     </row>
     <row r="51" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C51" s="14" t="s">
         <v>42</v>
@@ -3702,22 +3846,22 @@
         <v>43</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F51" s="14" t="s">
         <v>47</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H51" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J51" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K51" s="14" t="s">
         <v>142</v>
@@ -3737,10 +3881,10 @@
     </row>
     <row r="52" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C52" s="14" t="s">
         <v>50</v>
@@ -3749,22 +3893,22 @@
         <v>51</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F52" s="14" t="s">
         <v>52</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I52" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K52" s="14" t="s">
         <v>142</v>
@@ -3784,10 +3928,10 @@
     </row>
     <row r="53" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C53" s="14" t="s">
         <v>50</v>
@@ -3796,22 +3940,22 @@
         <v>43</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F53" s="14" t="s">
         <v>55</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I53" s="14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J53" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K53" s="14" t="s">
         <v>142</v>
@@ -3831,10 +3975,10 @@
     </row>
     <row r="54" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>50</v>
@@ -3843,22 +3987,22 @@
         <v>51</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F54" s="14" t="s">
         <v>59</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K54" s="14" t="s">
         <v>142</v>
@@ -3878,10 +4022,10 @@
     </row>
     <row r="55" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C55" s="14" t="s">
         <v>42</v>
@@ -3890,22 +4034,22 @@
         <v>43</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F55" s="14" t="s">
         <v>62</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I55" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K55" s="14" t="s">
         <v>142</v>
@@ -3925,10 +4069,10 @@
     </row>
     <row r="56" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C56" s="14" t="s">
         <v>29</v>
@@ -3937,22 +4081,22 @@
         <v>51</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H56" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I56" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K56" s="14" t="s">
         <v>142</v>
@@ -3972,10 +4116,10 @@
     </row>
     <row r="57" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C57" s="14" t="s">
         <v>42</v>
@@ -3984,22 +4128,22 @@
         <v>43</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F57" s="14" t="s">
         <v>68</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H57" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K57" s="14" t="s">
         <v>142</v>
@@ -4019,10 +4163,10 @@
     </row>
     <row r="58" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C58" s="14" t="s">
         <v>42</v>
@@ -4031,22 +4175,22 @@
         <v>43</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F58" s="14" t="s">
         <v>71</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I58" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K58" s="14" t="s">
         <v>142</v>

</xml_diff>